<commit_message>
Update: cleaned MISB101 entry in Excel file
</commit_message>
<xml_diff>
--- a/course_details.xlsx
+++ b/course_details.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mma/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mma/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{972FCB43-D70B-7843-91FF-E1DDE6076388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{216301D3-FF2E-8B4A-A45E-DD963E35C507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="740" windowWidth="35060" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15640" yWindow="1280" windowWidth="35060" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>